<commit_message>
feat: enhance UI aesthetics, implement batch execution tracking, manual SharePoint uploads, and fix button freeze, 404 upload, and download filename issues
</commit_message>
<xml_diff>
--- a/scratch/temp_output.xlsx
+++ b/scratch/temp_output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1072,12 +1072,12 @@
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
+      <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
@@ -1098,7 +1098,7 @@
       <c r="AO4" t="inlineStr"/>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>Mã sp NT03</t>
+          <t>NT03</t>
         </is>
       </c>
       <c r="AQ4" t="inlineStr"/>
@@ -1187,11 +1187,7 @@
           <t>Chờ xử lý</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
@@ -1216,11 +1212,7 @@
       <c r="AL5" t="inlineStr"/>
       <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>Tiêu cực</t>
-        </is>
-      </c>
+      <c r="AO5" t="inlineStr"/>
       <c r="AP5" t="inlineStr"/>
       <c r="AQ5" t="inlineStr"/>
     </row>

</xml_diff>